<commit_message>
Correcciones manuales verificadas contra los PDF y ajustes de clasificación
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contratacion_acuavalle_2024_2026.xlsx
+++ b/contratacion_acuavalle_2024_2026.xlsx
@@ -2205,7 +2205,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>accesorios, valvulas, almacen general</t>
+          <t>accesorios, valvulas, almacen general, repuestos</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -6781,12 +6781,10 @@
           <t>DEL CONTRATISTA: OBLIGACIONES©_ ESPECÍFICAS: El CONTRATISTA se obliga a cumplir este contrato en los términos aquí consignados —&gt; 16 comprometiéndose especificamente a lo siguiente: a). Ofrecer por cuenta de ACUAVALLE S.A.… • Presentar el informe del resultado de la subasta, e informes de sugerencia de precio base para los lotes sin postor. g). Recaudar depósitos previos del 20% correspondiente a la postura y saldo por adjudicaciones. h). Repetir… • Realizar de nuevo el procedimiento de subasta, en caso de que la totalidad de los bienes no hayan sido adjudicados previa autorización de la supervisión hasta que se logre la venta. Para tal efecto, se incluirá los bienes no… • Reembolsar a ACUAVALLE S.A. E.S.P., el producto de las ventas de los bienes, a los 20 días hábiles siguientes a la subasta, una vez descontada la comisión pactada y el IVA sobre la comisión, siempre y cuando el Adjudicatario…</t>
         </is>
       </c>
-      <c r="O66" s="2" t="n">
-        <v>25000000</v>
-      </c>
+      <c r="O66" s="2" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Solo cifras</t>
+          <t>Valor indeterminado (según el contrato)</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -6816,7 +6814,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>Fecha de firma tomada de la cláusula de suscripción</t>
+          <t>Fecha de firma tomada de la cláusula de suscripción; Campos corregidos manualmente (valor, valor_verificacion): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -7088,12 +7086,12 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Combustibles, vehículos y transporte</t>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>carrotanque</t>
+          <t>mantenimiento, abastecimiento de agua potable</t>
         </is>
       </c>
       <c r="T69" t="inlineStr">
@@ -7376,7 +7374,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -8532,12 +8530,12 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Materiales, tubería, accesorios y ferretería</t>
+          <t>Combustibles, vehículos y transporte</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>materiales, herramientas</t>
+          <t>vehiculo, vehiculos, llantas, transporte, transporte de personal</t>
         </is>
       </c>
       <c r="T84" t="inlineStr">
@@ -8997,10 +8995,12 @@
           <t>1). Desarrollar el objeto del Contrato y el cumplimiento del alcance, en las condiciones de calidad, oportunidad, y obligaciones definidas en el Contrato, el análisis de justificación, la invitación a ofertar y la propuesta… • Las demás inherentes a la naturaleza del contrato. I|</t>
         </is>
       </c>
-      <c r="O89" s="2" t="inlineStr"/>
+      <c r="O89" s="2" t="n">
+        <v>1898057746</v>
+      </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 1.898 en cifras y 1.898.057.746 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S92" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
@@ -11018,12 +11018,12 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>Combustibles, vehículos y transporte</t>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
         </is>
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>carrotanque</t>
+          <t>abastecimiento de agua potable</t>
         </is>
       </c>
       <c r="T110" t="inlineStr">
@@ -11249,21 +11249,29 @@
           <t>ACUAVALLE S.A. E.S.P.</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>CONSORCIO INTERVENTORIA SEVILLA 2025</t>
+        </is>
+      </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>Inicia con la suscripción del acta de inicio (acta no incluida en el documento publicado)</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>No consta en el documento</t>
-        </is>
-      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
@@ -11308,7 +11316,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/08/CONTRATO-DE-INTERVENTORIA-NRO-174-25.pdf</t>
         </is>
       </c>
-      <c r="V113" t="inlineStr"/>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (contratista, fecha_firma, fecha_inicio, fecha_fin): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11735,7 +11747,11 @@
           <t>800.174.842-3</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2025-05-23</t>
+        </is>
+      </c>
       <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
@@ -11798,7 +11814,7 @@
       </c>
       <c r="V118" t="inlineStr">
         <is>
-          <t>Contratista tomado del título del documento en el sitio web</t>
+          <t>Contratista tomado del título del documento en el sitio web; Campos corregidos manualmente (fecha_firma): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -11864,7 +11880,11 @@
         </is>
       </c>
       <c r="O119" s="2" t="inlineStr"/>
-      <c r="P119" t="inlineStr"/>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Valor por unidad: $440 por kg de chatarra vendida (sin valor total)</t>
+        </is>
+      </c>
       <c r="Q119" t="inlineStr">
         <is>
           <t>El pago se efectuará, previa elaboración de la factura electrónica por parte de ACUAVALLE S.A. E.S.P, la cual será entregada al COMPRADOR, quien deberá realizar la consignación respectiva en la cuenta corriente N* 80402607127 de Bancolombia a nombre de ACUAVALLE S.A. E.S.P. El pago se efectuará previa elaboración de la factura respectiva, generada por ACUAVALLE S.A. E.S.P. CLAUSULA</t>
@@ -11892,7 +11912,7 @@
       </c>
       <c r="V119" t="inlineStr">
         <is>
-          <t>ACUAVALLE actúa como VENDEDOR (venta de bienes); el contratista es el comprador; Valor no identificado en el texto OCR</t>
+          <t>ACUAVALLE actúa como VENDEDOR (venta de bienes); el contratista es el comprador; Campos corregidos manualmente (valor, valor_verificacion): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -12042,7 +12062,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>Tomado de letras</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -12068,7 +12088,7 @@
       </c>
       <c r="V121" t="inlineStr">
         <is>
-          <t>ACUAVALLE actúa como COMPRADOR; el contratista es el vendedor; No se identificaron obligaciones en el texto OCR</t>
+          <t>ACUAVALLE actúa como COMPRADOR; el contratista es el vendedor; Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026); No se identificaron obligaciones en el texto OCR</t>
         </is>
       </c>
     </row>
@@ -12078,7 +12098,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Contrato de compraventa</t>
+          <t>Contrato de promesa de compraventa</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -12129,8 +12149,14 @@
           <t>N2 Vez se verifique el cumplimiento ae lael _contrato será CÍÍÍÍÍÁ'JB T suecripeión en — as siguientes Condiciones pocl3 ACUAVALLE S.A, E.S.p. Pública de compraventa del inm Ueble a favOr de X… 7 SRNE 0 o — — — — — D 3 : ¡… • Registro _de la escritura ante la Oficina de Registro de Instrumentos Públicos correspond¡en.te, con constancia de que el predio fue debidamente transferido y se e - E lones pactadas y libres de ocupación • Presentación de la factura debi i S s : - éontl%actualmente aT e gzr;la&lt;;r:)t.e expedida y los demás documentos exigidos . . Certificación del Supervisor 1 O lec onesiper partepdel contrat?sí!a. contrato sobre el cumplimiento…</t>
         </is>
       </c>
-      <c r="O122" s="2" t="inlineStr"/>
-      <c r="P122" t="inlineStr"/>
+      <c r="O122" s="2" t="n">
+        <v>337920423</v>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Corregido manualmente (revisión del PDF)</t>
+        </is>
+      </c>
       <c r="Q122" t="inlineStr"/>
       <c r="R122" t="inlineStr">
         <is>
@@ -12139,7 +12165,7 @@
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>bien inmueble, predio, lote de terreno, derechos de dominio, posesion material, matricula inmobiliaria</t>
+          <t>tipo: contrato de promesa de compraventa, bien inmueble, predio, lote de terreno, derechos de dominio, posesion material</t>
         </is>
       </c>
       <c r="T122" t="inlineStr">
@@ -12154,7 +12180,7 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>ACUAVALLE actúa como COMPRADOR; el contratista es el vendedor; Valor no identificado en el texto OCR</t>
+          <t>ACUAVALLE actúa como COMPRADOR; el contratista es el vendedor; Campos corregidos manualmente (valor, tipo_documento): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12327,11 @@
         </is>
       </c>
       <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>ADQUIRIR AUTOMOTOR, TIPO CAMIONETA, DIÉSEL, TRACCION 4 X 2, MECÁNICA, PARA SER UTILIZADO EN ACTIVIDADES INSTITUCIONALES Y MISIONALES DE LA ENTIDAD</t>
+        </is>
+      </c>
       <c r="N124" t="inlineStr"/>
       <c r="O124" s="2" t="n">
         <v>194990000</v>
@@ -12318,10 +12348,14 @@
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>Sin clasificar (objeto no legible)</t>
-        </is>
-      </c>
-      <c r="S124" t="inlineStr"/>
+          <t>Combustibles, vehículos y transporte</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>diesel, camioneta</t>
+        </is>
+      </c>
       <c r="T124" t="inlineStr">
         <is>
           <t>Contratos de Compraventa</t>
@@ -12334,7 +12368,7 @@
       </c>
       <c r="V124" t="inlineStr">
         <is>
-          <t>ACUAVALLE actúa como COMPRADOR; el contratista es el vendedor; Objeto no identificado en el texto OCR; No se identificaron obligaciones en el texto OCR</t>
+          <t>ACUAVALLE actúa como COMPRADOR; el contratista es el vendedor; Campos corregidos manualmente (objeto): Revisión manual del PDF por el usuario (06/10/2026); No se identificaron obligaciones en el texto OCR</t>
         </is>
       </c>
     </row>
@@ -12692,7 +12726,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>Tomado de letras</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -12720,7 +12754,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/11/CONTRATO-DE-CONSULTORIA-NRO-142-25-DATEN-SAS.pdf</t>
         </is>
       </c>
-      <c r="V128" t="inlineStr"/>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -13359,10 +13397,12 @@
           <t>El documento solo contiene obligaciones de formato estándar (las mismas que se repiten en muchos contratos de Acuavalle); no se encontraron obligaciones específicas distintas</t>
         </is>
       </c>
-      <c r="O135" s="2" t="inlineStr"/>
+      <c r="O135" s="2" t="n">
+        <v>139699500</v>
+      </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -13372,7 +13412,7 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
@@ -13392,7 +13432,7 @@
       </c>
       <c r="V135" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 139.089.062 en cifras y 139.699.500 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -13554,7 +13594,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>Tomado de letras</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -13582,7 +13622,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/12/CONTRATO-DE-SUMINISTRO-NRO-166-25-CONTROL-E-INSTRUMENTACION-INDUSTRIAL-DE-COLOMBIA-SAS.pdf</t>
         </is>
       </c>
-      <c r="V137" t="inlineStr"/>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -13852,7 +13896,7 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
@@ -14145,7 +14189,7 @@
       </c>
       <c r="S143" t="inlineStr">
         <is>
-          <t>elementos electricos</t>
+          <t>elementos electricos, repuestos</t>
         </is>
       </c>
       <c r="T143" t="inlineStr">
@@ -14236,12 +14280,12 @@
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>Materiales, tubería, accesorios y ferretería</t>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
         </is>
       </c>
       <c r="S144" t="inlineStr">
         <is>
-          <t>herramientas</t>
+          <t>clorador</t>
         </is>
       </c>
       <c r="T144" t="inlineStr">
@@ -15911,21 +15955,29 @@
           <t>ACUAVALLE S.A. E.S.P.</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>FUNDACIÓN AMBIENTAL</t>
+        </is>
+      </c>
       <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
-      <c r="H162" t="inlineStr"/>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>Inicia con la suscripción del acta de inicio (acta no incluida en el documento publicado)</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr">
-        <is>
-          <t>No consta en el documento</t>
-        </is>
-      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr"/>
       <c r="M162" t="inlineStr">
         <is>
@@ -15966,7 +16018,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/08/CONTRATO-DE-OBRA-NRO-148-25.pdf</t>
         </is>
       </c>
-      <c r="V162" t="inlineStr"/>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (contratista, fecha_firma, fecha_inicio, fecha_fin): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -16432,10 +16488,14 @@
       </c>
       <c r="R167" t="inlineStr">
         <is>
-          <t>Otros</t>
-        </is>
-      </c>
-      <c r="S167" t="inlineStr"/>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>aforadores, limnimetric, rejillas</t>
+        </is>
+      </c>
       <c r="T167" t="inlineStr">
         <is>
           <t>Contratos de Obras</t>
@@ -16908,10 +16968,14 @@
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>Otros</t>
-        </is>
-      </c>
-      <c r="S172" t="inlineStr"/>
+          <t>Obras civiles en sedes, plantas y vías</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>locativ, sede administrativa</t>
+        </is>
+      </c>
       <c r="T172" t="inlineStr">
         <is>
           <t>Contratos de Obras</t>
@@ -17768,10 +17832,14 @@
       </c>
       <c r="R181" t="inlineStr">
         <is>
-          <t>Otros</t>
-        </is>
-      </c>
-      <c r="S181" t="inlineStr"/>
+          <t>Obras civiles en sedes, plantas y vías</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>locativ, sede administrativa</t>
+        </is>
+      </c>
       <c r="T181" t="inlineStr">
         <is>
           <t>Contratos de Obras</t>
@@ -22045,12 +22113,10 @@
           <t>El CONTRATISTA se obliga a cumplir este contrato en los términos aquí consignados comprometiéndose específicamente a lo siguiente: a). Ofrecer por cuenta de ACUAVALLE S.A. E.S.P. los bienes en el estado y sitio donde se… • Presentar el informe del resultado de la subasta, e informes de sugerencia de precio base para los lotes sin postor. g). Repetir el procedimiento de subasta en caso de que la totalidad de los bienes no hayan sido adjudicados,… • Reembolsar a ACUAVALLE S.A. E.S.P., el producto de las ventas de los bienes, a los 20 días hábiles siguientes a la subasta, una vez descontada la comisión pactada y el IVA sobre la comisión, siempre y cuando el Adjudicatario… • Reportar al supervisor, de manera inmediata, cualquier novedad o anomalía que pueda afectar la ejecución del contrato. k). Firmado el contrato por las partes, se elaborará la correspondiente acta de inicio, la cual estará…</t>
         </is>
       </c>
-      <c r="O226" s="2" t="n">
-        <v>35000000</v>
-      </c>
+      <c r="O226" s="2" t="inlineStr"/>
       <c r="P226" t="inlineStr">
         <is>
-          <t>Solo cifras</t>
+          <t>Valor indeterminado (según el contrato)</t>
         </is>
       </c>
       <c r="Q226" t="inlineStr"/>
@@ -22074,7 +22140,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/09/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-143-25-BANCO-POPULAR-SA.pdf</t>
         </is>
       </c>
-      <c r="V226" t="inlineStr"/>
+      <c r="V226" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (valor, valor_verificacion): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -24160,10 +24230,14 @@
       </c>
       <c r="R248" t="inlineStr">
         <is>
-          <t>Otros</t>
-        </is>
-      </c>
-      <c r="S248" t="inlineStr"/>
+          <t>Comunicaciones, publicidad y eventos</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>avisos</t>
+        </is>
+      </c>
       <c r="T248" t="inlineStr">
         <is>
           <t>Contratos de Prestación de Servicios</t>
@@ -24231,7 +24305,11 @@
           <t>EL PLAZO ESTABLECIDO PARA LA EJECUCIÓN DEL CONTRATO SERÁ HASTA EL 31 DE DICIEMBRE DE 2025; PLAZO CONTADO A PARTIR DE LA SUSCRIPCIÓN DEL ACTA DE INICIO QUE EN NINGÚN CASO PODRÁ SER ANTERIOR AL CUMPLIMIENTO DE LOS REQUISITOS DE EJECUCIÓN.</t>
         </is>
       </c>
-      <c r="M249" t="inlineStr"/>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>FABRICACION E INSTALACION DE PLATAFORMA PARA FACILITAR EL MANTENIMIENTO DE LAS UNIDADES DE AIRE ACONDICIONADO EN LA OFICINA PRINCIPAL DE ACUAVALLE S.A. E.S.P., EN EL DPTO DEL VALLE DEL CAUCA</t>
+        </is>
+      </c>
       <c r="N249" t="inlineStr">
         <is>
           <t>Ejecutar la programación de las actividades que debe desarrollar para el cumplimiento del objetivo del contrato • Garantizar la calidad del servicio • Garantizar óptimas relaciones interpersonales entre el personal a su cargo y el personal de las dependencias de la Entidad • Rendir y elaborar los informes que solicite el supervisor, conforme al objeto del contrato • Acatar las instrucciones que durante el desarrollo del contrato se le impartan por el Supervisor del contrato • Obrar con lealtad y buena fe en las diferentes etapas contractuales, evitando dilaciones y entrabamientos • Radicar las facturas de cobro por suministros o trabajos efectuados dentro de los plazos convenidos y según el avance de la ejecución contractual • Pago de la Seguridad Social de todo su equipo de trabajo (Salud, Pensión y Riesgos Laborales)</t>
@@ -24252,12 +24330,12 @@
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>Seguridad, salud en el trabajo y dotación</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>seguridad y salud, sst, elementos de proteccion, dotacion</t>
+          <t>aire acondicionado</t>
         </is>
       </c>
       <c r="T249" t="inlineStr">
@@ -24272,7 +24350,7 @@
       </c>
       <c r="V249" t="inlineStr">
         <is>
-          <t>Objeto no identificado en el texto OCR</t>
+          <t>Campos corregidos manualmente (objeto): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -25220,12 +25298,12 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>Combustibles, vehículos y transporte</t>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>carrotanque</t>
+          <t>abastecimiento de agua potable</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
@@ -26088,7 +26166,7 @@
       </c>
       <c r="R268" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S268" t="inlineStr">
@@ -27140,7 +27218,7 @@
       </c>
       <c r="R279" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S279" t="inlineStr">
@@ -27409,10 +27487,12 @@
           <t>Actuar con diligencia y respeto en el cumplimiento de sus obligaciones • Mantener el vehículo, en óptimas condiciones mecánicas, eléctricas, de tendido de llantas, aseo y presentación • Tener un seguro obligatorio de accidentes de tránsito vigente durante la vigencia del presente contrato • Tener las licencias de conducción vigente • Disponer de otro vehículo de las mismas características o similares, en forma temporal cuando el vehículo no pueda prestar el servicio por fallas mecánicas o accidente de tránsito, garantizando que igualmente esté amparado… • Presentar Certificado de Paz y Salvo por concepto de multas por infracciones de tránsito • El vehículo deberá estar dotado con todos los implementos necesarios para cubrir cualquier eventualidad, tales como: equipo de carretera completo (llantas de repuesto, herramientas, botiquín de primeros auxilios, extintor,… • El contratista deberá efectuar oportunamente y por su cuenta las reparaciones y el mantenimiento necesario al vehículo, tanto preventivo como correctivo y suministrar por cuenta propia los gastos inherentes a la prestación del…</t>
         </is>
       </c>
-      <c r="O282" s="2" t="inlineStr"/>
+      <c r="O282" s="2" t="n">
+        <v>118607500</v>
+      </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
@@ -27422,12 +27502,12 @@
       </c>
       <c r="R282" t="inlineStr">
         <is>
-          <t>Materiales, tubería, accesorios y ferretería</t>
+          <t>Combustibles, vehículos y transporte</t>
         </is>
       </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t>materiales, herramientas</t>
+          <t>vehiculo, vehiculos, llantas, transporte, transporte de personal</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
@@ -27442,7 +27522,7 @@
       </c>
       <c r="V282" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 118.607.500 en cifras y 125.607.500 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -28064,7 +28144,11 @@
         </is>
       </c>
       <c r="O289" s="2" t="inlineStr"/>
-      <c r="P289" t="inlineStr"/>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>Valor por unidad: $410 + IVA por kg de chatarra; el valor final depende del pesaje (estimado en el contrato: $2.460.000 + IVA por ~6.000 kg)</t>
+        </is>
+      </c>
       <c r="Q289" t="inlineStr">
         <is>
           <t>El pago se efectuará, previa elaboración de la factura electrónica por parte de ACUAVALLE S.A. E.S.P, la cual será entregada al COMPRADOR, quien deberá realizar la consignación respectiva en la cuenta corriente N% 80402607127 de Bancolombia a nombre de ACUAVALLE S.A. E.S.P. El pago se efectuará previa elaboración de la factura respectiva, generada por ACUAVALLE S.A. E.S.P. CLAUSULA</t>
@@ -28092,7 +28176,7 @@
       </c>
       <c r="V289" t="inlineStr">
         <is>
-          <t>ACUAVALLE actúa como VENDEDOR (venta de bienes); el contratista es el comprador; Valor no identificado en el texto OCR</t>
+          <t>ACUAVALLE actúa como VENDEDOR (venta de bienes); el contratista es el comprador; Campos corregidos manualmente (valor, valor_verificacion): Texto del contrato: cláusula cuarta (valor según pesaje) y consideraciones (precio mínimo por kg)</t>
         </is>
       </c>
     </row>
@@ -30001,7 +30085,7 @@
       </c>
       <c r="S309" t="inlineStr">
         <is>
-          <t>adecuaciones locativas, adecuacion</t>
+          <t>adecuaciones locativas, adecuacion, locativ, sede administrativa</t>
         </is>
       </c>
       <c r="T309" t="inlineStr">
@@ -30577,7 +30661,7 @@
       </c>
       <c r="S315" t="inlineStr">
         <is>
-          <t>adecuaciones locativas, oficinas administrativas, edificio, adecuacion</t>
+          <t>adecuaciones locativas, oficinas administrativas, edificio, adecuacion, locativ</t>
         </is>
       </c>
       <c r="T315" t="inlineStr">
@@ -34866,7 +34950,11 @@
         </is>
       </c>
       <c r="O360" s="2" t="inlineStr"/>
-      <c r="P360" t="inlineStr"/>
+      <c r="P360" t="inlineStr">
+        <is>
+          <t>Valor por unidad: $410 por kg de chatarra vendida (sin valor total)</t>
+        </is>
+      </c>
       <c r="Q360" t="inlineStr">
         <is>
           <t>El pago se efectuará, previa elaboración de la factura electrónica por parte de ACUAVALLE S.A. E.S.P, la cual será entregada al COMPRADOR, quien deberá realizar la consignación respectiva en la cuenta corriente N* 80402607127 de Bancolombia a nombre de ACUAVALLE S.A. E.S.P. El pago se efectuará previa elaboración de la factura respectiva, generada por ACUAVALLE S.A. E.S.P.. CLAUSULA</t>
@@ -34894,7 +34982,7 @@
       </c>
       <c r="V360" t="inlineStr">
         <is>
-          <t>ACUAVALLE actúa como VENDEDOR (venta de bienes); el contratista es el comprador; Valor no identificado en el texto OCR</t>
+          <t>ACUAVALLE actúa como VENDEDOR (venta de bienes); el contratista es el comprador; Campos corregidos manualmente (valor, valor_verificacion): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35203,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>SERCOMRED S.A.S . CEDULA O</t>
+          <t>SERCOMRED S.A.S</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
@@ -35155,10 +35243,12 @@
           <t>No aplica: el otrosí modifica valor y/o plazo del contrato principal</t>
         </is>
       </c>
-      <c r="O363" s="2" t="inlineStr"/>
+      <c r="O363" s="2" t="n">
+        <v>247333333</v>
+      </c>
       <c r="P363" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q363" t="inlineStr">
@@ -35188,7 +35278,7 @@
       </c>
       <c r="V363" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 247.333.333 en cifras y 33.333 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor, contratista): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -35268,12 +35358,12 @@
       </c>
       <c r="R364" t="inlineStr">
         <is>
-          <t>Bienestar, capacitación y talento humano</t>
+          <t>Obras civiles en sedes, plantas y vías</t>
         </is>
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t>capacitacion</t>
+          <t>locativ</t>
         </is>
       </c>
       <c r="T364" t="inlineStr">
@@ -37326,7 +37416,11 @@
       </c>
       <c r="N386" t="inlineStr"/>
       <c r="O386" s="2" t="inlineStr"/>
-      <c r="P386" t="inlineStr"/>
+      <c r="P386" t="inlineStr">
+        <is>
+          <t>Valor indeterminado (según el contrato)</t>
+        </is>
+      </c>
       <c r="Q386" t="inlineStr">
         <is>
           <t>El valor de la contraprestación estipulada en el presente contrato, se detraerá o descontará del dinero recaudado a favor del ALIADO COMERCIAL. El ingreso producto de la comisión pactada, se causará al momento de efectuar los giros con destino al ALIADO COMERCIAL.</t>
@@ -37334,12 +37428,12 @@
       </c>
       <c r="R386" t="inlineStr">
         <is>
-          <t>Materiales, tubería, accesorios y ferretería</t>
+          <t>Gestión comercial: lectura, facturación y atención a usuarios</t>
         </is>
       </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t>accesorios, materiales, medidores</t>
+          <t>servicio de facturacion</t>
         </is>
       </c>
       <c r="T386" t="inlineStr">
@@ -37354,7 +37448,7 @@
       </c>
       <c r="V386" t="inlineStr">
         <is>
-          <t>Contratista tomado del título del documento en el sitio web; Valor no identificado en el texto OCR; No se identificaron obligaciones en el texto OCR</t>
+          <t>Contratista tomado del título del documento en el sitio web; Campos corregidos manualmente (valor, valor_verificacion): Revisión manual del PDF por el usuario (06/10/2026); No se identificaron obligaciones en el texto OCR</t>
         </is>
       </c>
     </row>
@@ -37611,10 +37705,12 @@
           <t>I DEL CONTRATISTA: 1J Cum plir con el objeto del contrato en los térm inos aquí consignados • Presentar informes mensuales de actividades MdtFtorVbs proceso judicial • Representar a ACUAVALLE S.A E.S.P, de form a diligente y leal durante el trám ite de los procesos que se le asignen • Tener un archivo de todas las actuaciones de los procesos a su cargo • Sistem atizar la- Inform ación Referente a los procesos judiciales que se notifican en contra de la Entidad en el cuadro denominado Relación de Procesos, el cual sirve como guía para presentar los inform es por parte de la… • Realizar actividades.de acuerdo al objeto del presente contrato que le sean asignadas por la entidad contratante • Aceptar la revocatoria de cualquier poder o contrato de m andato entre el contratante y el contratista y verificar cada proceso de acuerdo a los informes presentados al supervisor • Revisar y estudiar las normas, conceptos, jurisprudencia y demás pronunciamientos de las autoridades representativas, relativos con el objeto y desempeño de ACUAVALLE S.A. E.S.P. a fin.de propender los procedimientos y…</t>
         </is>
       </c>
-      <c r="O389" s="2" t="inlineStr"/>
+      <c r="O389" s="2" t="n">
+        <v>92343133</v>
+      </c>
       <c r="P389" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q389" t="inlineStr">
@@ -37644,7 +37740,7 @@
       </c>
       <c r="V389" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 92.343.133 en cifras y 92.000.476 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -38578,7 +38674,7 @@
       </c>
       <c r="P399" t="inlineStr">
         <is>
-          <t>Tomado de letras</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q399" t="inlineStr">
@@ -38588,12 +38684,12 @@
       </c>
       <c r="R399" t="inlineStr">
         <is>
-          <t>Combustibles, vehículos y transporte</t>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
         </is>
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t>carrotanque</t>
+          <t>mantenimiento, abastecimiento de agua potable</t>
         </is>
       </c>
       <c r="T399" t="inlineStr">
@@ -38606,7 +38702,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/05/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-032-24-MR-INTEGRAL-GROUP-SAS.pdf</t>
         </is>
       </c>
-      <c r="V399" t="inlineStr"/>
+      <c r="V399" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -39060,7 +39160,7 @@
       </c>
       <c r="R404" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S404" t="inlineStr">
@@ -39325,10 +39425,12 @@
         </is>
       </c>
       <c r="N407" t="inlineStr"/>
-      <c r="O407" s="2" t="inlineStr"/>
+      <c r="O407" s="2" t="n">
+        <v>74700000</v>
+      </c>
       <c r="P407" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q407" t="inlineStr">
@@ -39358,7 +39460,7 @@
       </c>
       <c r="V407" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 74.700.000 en cifras y 74.000.700 en letras; requiere revisión del PDF; No se identificaron obligaciones en el texto OCR</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026); No se identificaron obligaciones en el texto OCR</t>
         </is>
       </c>
     </row>
@@ -39726,7 +39828,7 @@
       </c>
       <c r="R411" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S411" t="inlineStr">
@@ -40382,12 +40484,12 @@
       <c r="Q418" t="inlineStr"/>
       <c r="R418" t="inlineStr">
         <is>
-          <t>Materiales, tubería, accesorios y ferretería</t>
+          <t>Combustibles, vehículos y transporte</t>
         </is>
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t>materiales, herramientas</t>
+          <t>vehiculo, vehiculos, llantas, transporte, transporte de personal</t>
         </is>
       </c>
       <c r="T418" t="inlineStr">
@@ -41132,11 +41234,11 @@
         </is>
       </c>
       <c r="O426" s="2" t="n">
-        <v>116500000</v>
+        <v>50000000</v>
       </c>
       <c r="P426" t="inlineStr">
         <is>
-          <t>Solo cifras</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q426" t="inlineStr">
@@ -41164,7 +41266,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/12/OTROSI-NRO-1-ADICION-AL-CONTRATO-DE-SUMINISTRO-NRO-057-24-SUSCRITO-ENTRE-ACUAVALLE-SA-ESP-Y-INTEGRA-TIC-TECNOLOGIA-DE-OPTIMIZACION-SAS.pdf</t>
         </is>
       </c>
-      <c r="V426" t="inlineStr"/>
+      <c r="V426" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -41626,7 +41732,7 @@
       </c>
       <c r="R431" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="S431" t="inlineStr">
@@ -41707,10 +41813,12 @@
           <t>A.) DEL CONTRATISTA: Se obliga a cumplir este contrato en los términos aquí consignados comprometiéndose específicamente a lo siguiente • Entregar los suministros en el lugar, plazo y modo de acuerdo con el objeto del contrato • Tener buen trato y respeto con los usuarios y personal que labora en las dependencias de ACUAVALLE S.A. E.S.P • Suministrar por su cuenta y riesgo todo lo necesario para el cumplimiento del objeto contractual • Garantizar que su personal cuente con las herramientas adecuadas y las debidas precauciones de seguridad industrial tanto para su propia protección como para la de funcionarios y visitantes que se encuentren cercanos al área… • Transportar el insumo por su cuenta y riesgo, a los sitios donde se vayan a entregar el suministro, llevando consigo los equipos y herramientas que sean necesarios para ello • Atender adecuadamente las sugerencias y observaciones que hiciera ACUAVALLE S.A. E.S.P., a través de su Supervisor • Entregar oportunamente a ACUAVALLE S.A. E.S.P., los documentos que se exijan para garantizar el cumplimiento de lo estipulado, tales como Pólizas, Certificaciones y demás</t>
         </is>
       </c>
-      <c r="O432" s="2" t="inlineStr"/>
+      <c r="O432" s="2" t="n">
+        <v>67473000</v>
+      </c>
       <c r="P432" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q432" t="inlineStr">
@@ -41740,7 +41848,7 @@
       </c>
       <c r="V432" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 67.473.000 en cifras y 67.463.000 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -41906,7 +42014,7 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>Tomado de letras</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr">
@@ -41916,12 +42024,12 @@
       </c>
       <c r="R434" t="inlineStr">
         <is>
-          <t>Asesoría jurídica, financiera y auditoría</t>
+          <t>Mantenimiento, operación y automatización de sistemas</t>
         </is>
       </c>
       <c r="S434" t="inlineStr">
         <is>
-          <t>abogado, tributari</t>
+          <t>clorador</t>
         </is>
       </c>
       <c r="T434" t="inlineStr">
@@ -41934,7 +42042,11 @@
           <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/10/CONTRATO-DE-SUMINISTRO-NRO-100-24-REGAL-SYSTEMS-COLOMBIA-SAS.pdf</t>
         </is>
       </c>
-      <c r="V434" t="inlineStr"/>
+      <c r="V434" t="inlineStr">
+        <is>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="n">
@@ -43049,10 +43161,12 @@
           <t>E n E , DEL VALLE DEL CAUCA S.A. E.S.P, tyº' ACUAVALLE S.A. E.S.P. A Més Por Ves CONTRATO DE SUMINISTRO No. 047-24 • Suministro de materiales de excelente calidad, como son: areña, triturado, cemento, sika secante, hierro, alambre • Garantizar la calidad de los insumos suministrados, por el término estipulado, contados a partir de la entrega de los mismos • A realizar el suministro conforme a todas las especificaciones ofrecidas y en los términos pactados, • Contratar por su cuenta y riesgo, . con plena autonomia para ello, el personal necesario o conveniente para la ejecución del contrato • Presentar los soportes que garanticen la entrega de los suministros • Transportar loes insumes desde la planta de producción hasta el sitio de entrega por su cuenta y riesgo • Garantizar la calidad de los materiales solicitados</t>
         </is>
       </c>
-      <c r="O446" s="2" t="inlineStr"/>
+      <c r="O446" s="2" t="n">
+        <v>96280000</v>
+      </c>
       <c r="P446" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q446" t="inlineStr">
@@ -43082,7 +43196,7 @@
       </c>
       <c r="V446" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 96.280.000 en cifras y 96.000.280 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -44487,10 +44601,12 @@
           <t>Realizar los diseños definitivos e ingeniería de detalle de los componentes requeridos para dar cumplimiento al alcance del objeto, en función de la normatividad actual y las nuevas disposiciones que la complementen o… • Presentar mensualmente un informe de actividades con su respectiva presentación en formato Microsoft Power Point o PDF, para verificar y hacer seguimiento al cumplimiento de la Metodología de Trabajo y al cronograma acordado… • Responder por cualquier tipo de reclamación judicial o — extrajudicial que instaure, impulse o en la que coadyuve su personal o sus subcontratistas con ACUAVALLE S.A E.S.P., por causa o con ocasión del contrato. h),, &gt; ())y J…</t>
         </is>
       </c>
-      <c r="O461" s="2" t="inlineStr"/>
+      <c r="O461" s="2" t="n">
+        <v>1455816250</v>
+      </c>
       <c r="P461" t="inlineStr">
         <is>
-          <t>Pendiente de revisión manual (cifras ≠ letras)</t>
+          <t>Corregido manualmente (revisión del PDF)</t>
         </is>
       </c>
       <c r="Q461" t="inlineStr">
@@ -44520,7 +44636,7 @@
       </c>
       <c r="V461" t="inlineStr">
         <is>
-          <t>Valor no incluido en totales: el OCR leyó 1.455.816.250 en cifras y 2.455.816.250 en letras; requiere revisión del PDF</t>
+          <t>Campos corregidos manualmente (valor): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -44769,8 +44885,14 @@
           <t>Actuar con diligencia, honestidad y 6 e, ACUAVALLE respeto en el cumplimiento de sus obligaciones.3) Evaluar el plan de seguros que actualmente tiene ACUAVALLE S.A. E.S.P., examinando las condiciones de riesgos y asesoría en… • Asesorar, presentar y tramitar en forma oportuna las reclamaciones de _ siniestros ante las aseguradoras y procurar obtener indemnizaciones que correspondan en las mejores condiciones de modo, tiempo y cuantía • Presentar asesoría en evaluación y análisis de riesgos, diseñando un programa de administración para este efecto.10) Informar acerca de las decisiones adoptadas por la Superintendencia Financiera de Colombia en materia de… • Ofrecer servicios especiales a ACUAVALLE S.A. E.S.P., para atender concretamente su programa de seguros, presentando beneficios económicos, técnicos o administrativos • Prestar todos los demás servicios que emanan de la actividad de Intermediación de Seguros y todas aquellas que señale la Constitución Política y la Ley.15) Obrar con lealtad y buena fe en las distintas etapas contractuales,… • No acceder a peticiones o amenazas de quien actúe por fuera de la ley con el fin de obligarlos a hacer u omitir algún acto o hecho.17) Prestar con recursos humanos, técnicos y logísticos propios, la asesoría e intermediación…</t>
         </is>
       </c>
-      <c r="O464" s="2" t="inlineStr"/>
-      <c r="P464" t="inlineStr"/>
+      <c r="O464" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P464" t="inlineStr">
+        <is>
+          <t>No genera erogación para Acuavalle</t>
+        </is>
+      </c>
       <c r="Q464" t="inlineStr">
         <is>
           <t>El contrato de Intermediación de Seguros, no causa erogación alguna para ACUAVALLE S.A. E.S.P., por lo cual no requiere disponibilidad presupuestal, y cualquier pago que genere la intermediación será por cuenta de la(s) compañía(s) de seguros con la(s) que se suscriban las pólizas. .SEXTA. -SUJECION DE LOS PAGOS A LAS APROPIACIONES PRESUPUESTALES: El contrato que resulte del presente proceso de selección no genera…</t>
@@ -44798,7 +44920,7 @@
       </c>
       <c r="V464" t="inlineStr">
         <is>
-          <t>Valor no identificado en el texto OCR</t>
+          <t>Campos corregidos manualmente (valor, valor_verificacion): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -44927,7 +45049,11 @@
           <t>800.174.842-3</t>
         </is>
       </c>
-      <c r="G466" t="inlineStr"/>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>2024-08-22</t>
+        </is>
+      </c>
       <c r="H466" t="inlineStr"/>
       <c r="I466" t="inlineStr">
         <is>
@@ -44990,7 +45116,7 @@
       </c>
       <c r="V466" t="inlineStr">
         <is>
-          <t>Contratista tomado del título del documento en el sitio web</t>
+          <t>Contratista tomado del título del documento en el sitio web; Campos corregidos manualmente (fecha_firma): Revisión manual del PDF por el usuario (06/10/2026)</t>
         </is>
       </c>
     </row>
@@ -45473,7 +45599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -45516,10 +45642,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>28821697202</v>
+        <v>32369215229</v>
       </c>
     </row>
     <row r="4">
@@ -45545,33 +45671,33 @@
         <v>40</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24214180341</v>
+        <v>24395013674</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gestión comercial: lectura, facturación y atención a usuarios</t>
+          <t>Vigilancia, aseo, mobiliario y servicios generales</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>13627157167</v>
+        <v>13844372692</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Vigilancia, aseo y servicios generales</t>
+          <t>Gestión comercial: lectura, facturación y atención a usuarios</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>13615423192</v>
+        <v>13627157167</v>
       </c>
     </row>
     <row r="8">
@@ -45584,7 +45710,7 @@
         <v>16</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>12809502528</v>
+        <v>12876975528</v>
       </c>
     </row>
     <row r="9">
@@ -45610,7 +45736,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>7193769892</v>
+        <v>8649586142</v>
       </c>
     </row>
     <row r="11">
@@ -45620,36 +45746,36 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7042412836</v>
+        <v>6694262684</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Combustibles, vehículos y transporte</t>
+          <t>Gestión ambiental y cuencas</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>5359494613</v>
+        <v>4780775564</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gestión ambiental y cuencas</t>
+          <t>Combustibles, vehículos y transporte</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>4780775564</v>
+        <v>4667224880</v>
       </c>
     </row>
     <row r="14">
@@ -45659,75 +45785,75 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3238420169</v>
+        <v>3330060618</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laboratorio y control de calidad del agua</t>
+          <t>Obras civiles en sedes, plantas y vías</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2722936827</v>
+        <v>2727231112</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Obras civiles en sedes, plantas y vías</t>
+          <t>Laboratorio y control de calidad del agua</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2067536334</v>
+        <v>2722936827</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Seguridad, salud en el trabajo y dotación</t>
+          <t>Comunicaciones, publicidad y eventos</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1863658030</v>
+        <v>1890115080</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Servicios bancarios y recaudo</t>
+          <t>Seguridad, salud en el trabajo y dotación</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1660983274</v>
+        <v>1774408030</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Comunicaciones, publicidad y eventos</t>
+          <t>Servicios bancarios y recaudo</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
         <v>6</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1611260000</v>
+        <v>1660983274</v>
       </c>
     </row>
     <row r="20">
@@ -45737,23 +45863,23 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>985000952</v>
+        <v>821554452</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Compra de predios e inmuebles</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
         <v>4</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>898863570</v>
+        <v>766854640</v>
       </c>
     </row>
     <row r="22">
@@ -45772,53 +45898,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Compra de predios e inmuebles</t>
+          <t>Arrendamiento de inmuebles</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>428934217</v>
+        <v>70930693</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sin clasificar (objeto no legible)</t>
+          <t>Venta de bienes dados de baja (ingreso)</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>194990000</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Arrendamiento de inmuebles</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>70930693</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Venta de bienes dados de baja (ingreso)</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>60000000</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -45909,7 +46009,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4721888861</v>
+        <v>6177705111</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>1177029049</v>
@@ -45957,13 +46057,13 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>31121941526</v>
+        <v>31288984659</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>38280044196</v>
+        <v>38363651696</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45653110623</v>
+        <v>47526168369</v>
       </c>
     </row>
     <row r="9">
@@ -45976,7 +46076,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>355538617</v>
+        <v>693459040</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
@@ -45989,10 +46089,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>7443528036</v>
+        <v>7607281036</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>8579823759</v>
+        <v>8719523259</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>7386703588</v>
@@ -46021,7 +46121,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>553500000</v>
+        <v>734333333</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>0</v>
@@ -46041,7 +46141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -46090,1011 +46190,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>110-26</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>BANCO POPULARSA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (solo cifras)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/10/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-110-26-BANCO-POPULAR-SA.pdf</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>f1ea0860</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>054-26</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SOLUCIONES AUTOMATICAS PROGRAMABLES S.A.P. SAS</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 1.898 en cifras y 1.898.057.746 en letras)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/03/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-054-26-SOLUCIONES-AUTOMATICAS-PROGRAMABLES-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2f69ef50</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>174-25</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Contrato de interventoría</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Fecha de firma no legible</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>158321506</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/08/CONTRATO-DE-INTERVENTORIA-NRO-174-25.pdf</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>855b3b42</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>001-2025</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Convenio interadministrativo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CORPOCUENCAS</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Fecha de firma no legible</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>303402200</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/05/Convenio-Interadministrativo-No.-001-2025-Celebrado-Entre-ACUAVALLE-SA-ESP-y-CORPOCUENCAS.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>974e0307</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>146-25</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Contrato de compraventa</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EMPRESA COLOMBIANA DE ASEO S.A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Valor no legible en el OCR</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/09/CONTRATO-DE-COMPRAVENTA-NRO-146-25-EMPRESA-COLOMBIANA-DE-ASEO-SA.pdf</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>87117a5e</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>160-25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Contrato de promesa de compraventa</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>BETTY GUILLERMINA ORTIZ MAFLA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (tomado de letras)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>355538617</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/12/CONTRATO-DE-PROMESA-DE-COMPRAVENTA-DE-BIEN-INMUEBLE-NRO-160-25-BETTY-GUILLERMINA-ORTIZ-MAFLA.pdf</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>1a7f3f58</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>135-25</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Contrato de compraventa</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CONSTRUCTORA GRAM HABITAT S.A</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Valor no legible en el OCR</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/12/CONTRATO-COMPRA-VENTA-NRO-135-25-CONSTRUCTORA-GRAM-HABITAT-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>8a23c5f5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>043-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Contrato de compraventa</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>AUTOPACIFICO S.A</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Objeto no legible</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>194990000</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/04/CONTRATO-DE-COMPRAVENTA-DE-BIEN-INMUEBLE-NRO-043-25-AUTOPACIFICO-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>30acceb4</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>142-25</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Contrato de consultoría</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DATEN S.A.S</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (tomado de letras)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>86781401</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/11/CONTRATO-DE-CONSULTORIA-NRO-142-25-DATEN-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>c14eb5c9</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>156-25</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Contrato de suministro</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>DANIELA ANDREA COSTA GÓMEZ</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 139.089.062 en cifras y 139.699.500 en letras)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/02/CONTRATO-DE-SUMINISTRO-NRO-156-25-DANIELA-ANDREA-COSTA-GOMEZ.pdf</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>b141ff54</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>166-25</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Contrato de suministro</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>CONTROL E INSTRUMENTACIÓN INDUSTRIAL DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (tomado de letras)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>265996832</v>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/12/CONTRATO-DE-SUMINISTRO-NRO-166-25-CONTROL-E-INSTRUMENTACION-INDUSTRIAL-DE-COLOMBIA-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>343a5d9b</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>148-25</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Contrato de obra</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Fecha de firma no legible</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>2098977636</v>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/08/CONTRATO-DE-OBRA-NRO-148-25.pdf</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>836b9c2d</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>143-25</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>BANCO POPULAR S.A</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (solo cifras)</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2026/09/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-143-25-BANCO-POPULAR-SA.pdf</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>ec875b3f</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>110-25</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>ALQUIMIA 2.0 S.A.S</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Objeto no legible</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>89250000</v>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/08/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-110-25-ALQUIMIA-2.0-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>02e28fc1</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>005-25</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>OLVIN TORRES RIVERA</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 118.607.500 en cifras y 125.607.500 en letras)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/02/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-005-25-OLVIN-TORRES-RIVERA.pdf</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>6aac4472</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Contrato de compraventa</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>EMPRESA COLOMBIANA DE ASEO S.A</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Valor no legible en el OCR</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/01/CONTRATO-DE-COMPRAVENTA-EMPRESA-COLOMBIANA-DE-ASEO-SA.pdf</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>90a9d0ec</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>018-24</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Contrato de compraventa</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>EMPRESA COLOMBIANA DE ASEO S.A</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Valor no legible en el OCR</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/03/CONTRATO-DE-COMPRAVENTA-NRO-018-24-EMPRESA-COLOMBIANA-DE-ASEO-SA.pdf</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>cf83106b</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Otrosí 1 al contrato 009-24</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Otrosí / modificación</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>SERCOMRED S.A.S . CEDULA O</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 247.333.333 en cifras y 33.333 en letras)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2025/01/OTROSI-NRO-1-ADICION-Y-PROROGA-AL-CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-009-24-SUSCRITO-ENTRE-ACUAVALLE-SA-ESP-Y-SERVICIOS-EN-COMUNICACIONES-Y-REDES-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>de92ccd4</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>076-24</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>SERVICOMERCIAL DE TULUÁ SAS</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Valor no legible en el OCR</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/08/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-076-24-SERVICOMERCIAL-DE-TULUA-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>26c6b7e7</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>008-24</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GONZALO MANRIQUE ZULUAGA</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 92.343.133 en cifras y 92.000.476 en letras)</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/06/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-008-24-GONZALO-MANRIQUE-ZULUAGA.pdf</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>8cd57f94</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>032-24</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MRINTEGRAL GROUP S.A.S</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (tomado de letras)</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>258316064</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/05/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-032-24-MR-INTEGRAL-GROUP-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>acbabfb3</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>037-24</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Contrato de prestación de servicios</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MARIA CAMILA REYES ROMERO</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 74.700.000 en cifras y 74.000.700 en letras)</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/04/CONTRATO-DE-PRESTACION-DE-SERVICIOS-NRO-037-24-MARIA-CAMILA-REYES-ROMERO.pdf</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>df7c25f3</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Otrosí 1 al contrato 057-24</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Otrosí / modificación</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>INTEGRA TIC TECNOLOGÍA DE OPTIMIZACIÓN SAS</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (solo cifras)</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>116500000</v>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/12/OTROSI-NRO-1-ADICION-AL-CONTRATO-DE-SUMINISTRO-NRO-057-24-SUSCRITO-ENTRE-ACUAVALLE-SA-ESP-Y-INTEGRA-TIC-TECNOLOGIA-DE-OPTIMIZACION-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>d533181e</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>095-24</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Contrato de suministro</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>PROFINAS S.A.S</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 67.473.000 en cifras y 67.463.000 en letras)</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/10/CONTRATO-DE-SUMINISTRO-NRO-095-24-PROFINAS-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>19cbd7d9</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>100-24</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Contrato de suministro</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>REGAL SYSTEMS COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Valor sin doble verificación (tomado de letras)</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>75402684</v>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/10/CONTRATO-DE-SUMINISTRO-NRO-100-24-REGAL-SYSTEMS-COLOMBIA-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>a3aaaf07</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>047-24</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Contrato de suministro</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>DIEGO HUMBERTO PEREZ VILLAFANE</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 96.280.000 en cifras y 96.000.280 en letras)</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/06/CONTRATO-DE-SUMINISTRO-NRO-047-24-DIEGO-HUMBERTO-PEREZ-VILLAFANE.pdf</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>388e158e</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>090-24</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Contrato de consultoría</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>GRUPO IGEI S.A.S</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Valor: cifras ≠ letras (OCR leyó 1.455.816.250 en cifras y 2.455.816.250 en letras)</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/09/CONTRATO-DE-CONSULTORIA-NRO-090-24-GRUPO-IGEI-SAS.pdf</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>d9690b11</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>050-24</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Contrato de consultoría</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>GONSEGUROS CORREDORES DE SEGUROS S.A</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Valor no legible en el OCR</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/05/CONTRATO-DE-COSULTORIA-NRO-050-24-GONSEGUROS-CORREDORES-DE-SEGUROS-SA.pdf</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>5e8bd2c2</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>NRO-003-2024</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Convenio interadministrativo</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>CORPOCUENCAS</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Fecha de firma no legible</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>302480000</v>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>https://www.acuavalle.gov.co/wp-content/uploads/2024/08/CONVENIO-INTRERADMINISTRATIVO-NRO-003-2024-CORPOCUENCAS.pdf</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>a0ace4cc</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId29"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>